<commit_message>
Rebuild dos artefatos do Guia
</commit_message>
<xml_diff>
--- a/Guia_de_Ofertas_Tratado_para_Validacao_V2_Escopo_Ampliado.xlsx
+++ b/Guia_de_Ofertas_Tratado_para_Validacao_V2_Escopo_Ampliado.xlsx
@@ -70199,7 +70199,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -70233,9 +70233,10 @@
       <c r="A4" s="10" t="s">
         <v>2155</v>
       </c>
-      <c r="B4" s="16">
-        <f>COUNTA('Fluxos Tratados'!A2:A115)</f>
-        <v>114</v>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
       </c>
       <c r="C4" s="10" t="s">
         <v>2156</v>
@@ -70245,9 +70246,10 @@
       <c r="A5" s="10" t="s">
         <v>2157</v>
       </c>
-      <c r="B5" s="16">
-        <f>COUNTIF('Fluxos Tratados'!V2:V115,"ADEQUADO")</f>
-        <v>8</v>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="C5" s="10" t="s">
         <v>2158</v>
@@ -70287,9 +70289,10 @@
       <c r="A8" s="10" t="s">
         <v>2163</v>
       </c>
-      <c r="B8" s="16">
-        <f>COUNTIF('Fluxos Tratados'!V2:V115,"PENDENTE")</f>
-        <v>21</v>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
       </c>
       <c r="C8" s="10" t="s">
         <v>2164</v>
@@ -70432,7 +70435,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
@@ -70527,8 +70530,10 @@
       <c r="B7" s="10" t="s">
         <v>2198</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>2209</v>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>85 registros A VALIDAR e itens adicionais por recurso/base normativa na aba de pendências.</t>
+        </is>
       </c>
       <c r="D7" s="10" t="s">
         <v>2210</v>
@@ -70544,14 +70549,20 @@
       <c r="B8" s="10" t="s">
         <v>2198</v>
       </c>
-      <c r="C8" s="10" t="s">
-        <v>2213</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>2214</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>2215</v>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>0 registros NÃO MAPEADO e 21 registros PENDENTE. Os 26 casos antes classificados como NÃO MAPEADO foram reclassificados para A VALIDAR após a revisão do escopo ampliado.</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Revisar A VALIDAR/PENDENTE</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>As reclassificações permanecem sujeitas à validação técnica quando a equivalência não é definitiva.</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:5" ht="43.5">
@@ -70612,8 +70623,10 @@
       <c r="A14" s="10" t="s">
         <v>2226</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>2227</v>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>A estrutura e a rastreabilidade estão adequadas, mas permanecem 85 registros A VALIDAR, 21 PENDENTE e lacunas de base normativa que exigem decisão do departamento e/ou atualização do Banco Mestre.</t>
+        </is>
       </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>

</xml_diff>